<commit_message>
Added plots of relative abundance of trace element species
</commit_message>
<xml_diff>
--- a/Zinc/6. Statistical data analysis/Typology_Date Interaction/interaction_results.xlsx
+++ b/Zinc/6. Statistical data analysis/Typology_Date Interaction/interaction_results.xlsx
@@ -38,13 +38,13 @@
     <t xml:space="preserve">Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Date:TypologyNP Tribs</t>
-  </si>
-  <si>
     <t xml:space="preserve">Date:TypologyP Tribs</t>
   </si>
   <si>
     <t xml:space="preserve">Date:TypologyPD Tribs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:TypologyMain Stem</t>
   </si>
   <si>
     <t xml:space="preserve">log_DOC_nM</t>
@@ -428,13 +428,13 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>10.92235348977</v>
+        <v>14.4278863638996</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00186921682888618</v>
+        <v>0.0996185006686501</v>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -445,10 +445,10 @@
         <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.00000000176111392156237</v>
+        <v>-0.00000000422303922898637</v>
       </c>
       <c r="D3" t="n">
-        <v>0.386468824878702</v>
+        <v>0.40952281246759</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -462,10 +462,10 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.00000000246192530742715</v>
+        <v>0.00000000477766390154945</v>
       </c>
       <c r="D4" t="n">
-        <v>0.654869196105432</v>
+        <v>0.388800575814765</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -479,10 +479,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00000000231573859412653</v>
+        <v>0.00000000876962127638365</v>
       </c>
       <c r="D5" t="n">
-        <v>0.43096213459221</v>
+        <v>0.11019890612616</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -496,13 +496,13 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0000000063076959689589</v>
+        <v>0.00000000246192530742419</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0259885146931955</v>
+        <v>0.654869196105862</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -513,13 +513,13 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>4.56768000983495</v>
+        <v>8.68077820589177</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0487469599908048</v>
+        <v>0.134796901780135</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.00000000044140294305774</v>
+        <v>-0.00000000212326523260602</v>
       </c>
       <c r="D8" t="n">
-        <v>0.743160790539798</v>
+        <v>0.531447196529573</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -547,10 +547,10 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.00000000256466817565917</v>
+        <v>-0.00000000111762423420975</v>
       </c>
       <c r="D9" t="n">
-        <v>0.482382460799296</v>
+        <v>0.760879844815009</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -564,10 +564,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.00000000368229240987496</v>
+        <v>0.000000000918868315461461</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0593553512867249</v>
+        <v>0.800282972094896</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -581,10 +581,10 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.00000000164579986020168</v>
+        <v>0.00000000256466817566442</v>
       </c>
       <c r="D11" t="n">
-        <v>0.379316280894751</v>
+        <v>0.482382460798459</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -598,13 +598,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>8.07921898094633</v>
+        <v>2.38009870920957</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0000000000754716543090559</v>
+        <v>0.430521753982109</v>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -615,10 +615,10 @@
         <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.000000000950200191859856</v>
+        <v>0.00000000184296048916391</v>
       </c>
       <c r="D13" t="n">
-        <v>0.176096505126052</v>
+        <v>0.297145716986066</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -632,10 +632,10 @@
         <v>8</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00000000279316068101697</v>
+        <v>-0.0000000029355752697789</v>
       </c>
       <c r="D14" t="n">
-        <v>0.142261128657119</v>
+        <v>0.125391983486441</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -649,10 +649,10 @@
         <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.000000000142414588754376</v>
+        <v>-0.00000000360071669322087</v>
       </c>
       <c r="D15" t="n">
-        <v>0.88834629561426</v>
+        <v>0.0575822691516285</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -666,10 +666,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.000000000807556012196928</v>
+        <v>-0.00000000279316068102493</v>
       </c>
       <c r="D16" t="n">
-        <v>0.407415055013369</v>
+        <v>0.142261128656032</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -683,10 +683,10 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.402581703993623</v>
+        <v>8.05404382257462</v>
       </c>
       <c r="D17" t="n">
-        <v>0.86361556118397</v>
+        <v>0.17110955523602</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -700,13 +700,13 @@
         <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>0.00000000354627324598913</v>
+        <v>-0.00000000193459872463821</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00977002482686196</v>
+        <v>0.573887682211506</v>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -717,10 +717,10 @@
         <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.00000000548087197062552</v>
+        <v>0.00000000370719949639746</v>
       </c>
       <c r="D19" t="n">
-        <v>0.139228498282643</v>
+        <v>0.319807741474092</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -734,10 +734,10 @@
         <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.00000000177367247423047</v>
+        <v>0.00000000424904569130217</v>
       </c>
       <c r="D20" t="n">
-        <v>0.36948557789625</v>
+        <v>0.249071628715834</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -751,10 +751,10 @@
         <v>10</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.00000000123182627932569</v>
+        <v>0.0000000054808719706282</v>
       </c>
       <c r="D21" t="n">
-        <v>0.516285693745441</v>
+        <v>0.139228498282502</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -768,13 +768,13 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>6.74814520173774</v>
+        <v>2.02518072560041</v>
       </c>
       <c r="D22" t="n">
-        <v>0.000000278531065087939</v>
+        <v>0.530959673727395</v>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -785,10 +785,10 @@
         <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.000000000355500764405498</v>
+        <v>0.00000000181525733750034</v>
       </c>
       <c r="D23" t="n">
-        <v>0.63602537732965</v>
+        <v>0.337468429933007</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -802,10 +802,10 @@
         <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>0.00000000217075810190854</v>
+        <v>-0.00000000167301214034345</v>
       </c>
       <c r="D24" t="n">
-        <v>0.286478962943363</v>
+        <v>0.414103890077232</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -819,10 +819,10 @@
         <v>9</v>
       </c>
       <c r="C25" t="n">
-        <v>0.000000000497745961561959</v>
+        <v>-0.00000000251292154086243</v>
       </c>
       <c r="D25" t="n">
-        <v>0.646797137507039</v>
+        <v>0.215156931471842</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -836,10 +836,10 @@
         <v>10</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.000000000342163438955637</v>
+        <v>-0.00000000217075810190554</v>
       </c>
       <c r="D26" t="n">
-        <v>0.742938239240848</v>
+        <v>0.286478962944091</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -853,13 +853,13 @@
         <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>5.05856787192688</v>
+        <v>0.785417648386047</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0000115877245112108</v>
+        <v>0.783076551909004</v>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -870,10 +870,10 @@
         <v>7</v>
       </c>
       <c r="C28" t="n">
-        <v>0.00000000036613574567506</v>
+        <v>0.00000000241175397344075</v>
       </c>
       <c r="D28" t="n">
-        <v>0.580879255703697</v>
+        <v>0.149203173260874</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -887,10 +887,10 @@
         <v>8</v>
       </c>
       <c r="C29" t="n">
-        <v>0.000000002045618227766</v>
+        <v>0.0000000000314561698215369</v>
       </c>
       <c r="D29" t="n">
-        <v>0.255264802511187</v>
+        <v>0.986115465995137</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -904,13 +904,13 @@
         <v>9</v>
       </c>
       <c r="C30" t="n">
-        <v>0.00000000207707439758722</v>
+        <v>-0.00000000316641299153383</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0308465973539595</v>
+        <v>0.0771975386732452</v>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -921,10 +921,10 @@
         <v>10</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.00000000112079476376756</v>
+        <v>-0.00000000204561822776544</v>
       </c>
       <c r="D31" t="n">
-        <v>0.224094480728658</v>
+        <v>0.255264802511379</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -938,10 +938,10 @@
         <v>6</v>
       </c>
       <c r="C32" t="n">
-        <v>3.59886906706793</v>
+        <v>7.04248087966967</v>
       </c>
       <c r="D32" t="n">
-        <v>0.161457115033839</v>
+        <v>0.274265168538103</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -955,10 +955,10 @@
         <v>7</v>
       </c>
       <c r="C33" t="n">
-        <v>0.00000000100810988213973</v>
+        <v>-0.0000000015968881926404</v>
       </c>
       <c r="D33" t="n">
-        <v>0.500494897313527</v>
+        <v>0.671653314622946</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -972,10 +972,10 @@
         <v>8</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.00000000260499807477768</v>
+        <v>0.00000000387430684354268</v>
       </c>
       <c r="D34" t="n">
-        <v>0.520518138376013</v>
+        <v>0.342409646563053</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -989,10 +989,10 @@
         <v>9</v>
       </c>
       <c r="C35" t="n">
-        <v>0.00000000126930876876204</v>
+        <v>0.00000000242121137951254</v>
       </c>
       <c r="D35" t="n">
-        <v>0.557452872129296</v>
+        <v>0.548418359666595</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1006,10 +1006,10 @@
         <v>10</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.000000000183786695267869</v>
+        <v>0.00000000260499807478064</v>
       </c>
       <c r="D36" t="n">
-        <v>0.929516334375837</v>
+        <v>0.520518138375593</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1023,10 +1023,10 @@
         <v>6</v>
       </c>
       <c r="C37" t="n">
-        <v>3.04744296276921</v>
+        <v>5.17232642376286</v>
       </c>
       <c r="D37" t="n">
-        <v>0.121544923929286</v>
+        <v>0.294186005022538</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1040,10 +1040,10 @@
         <v>7</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0000000015653596256314</v>
+        <v>-0.000000000239999989235766</v>
       </c>
       <c r="D38" t="n">
-        <v>0.172204930124245</v>
+        <v>0.93366932437823</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1057,10 +1057,10 @@
         <v>8</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.00000000180535961486482</v>
+        <v>-0.000000000496359136490603</v>
       </c>
       <c r="D39" t="n">
-        <v>0.560744173836638</v>
+        <v>0.873675638315646</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1074,10 +1074,10 @@
         <v>9</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.00000000230171875135804</v>
+        <v>0.00000000131386807545057</v>
       </c>
       <c r="D40" t="n">
-        <v>0.165130821294631</v>
+        <v>0.67049789711735</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1091,10 +1091,10 @@
         <v>10</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.000000000491491539416585</v>
+        <v>0.00000000180535961486761</v>
       </c>
       <c r="D41" t="n">
-        <v>0.757336426606069</v>
+        <v>0.560744173836084</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1108,13 +1108,13 @@
         <v>6</v>
       </c>
       <c r="C42" t="n">
-        <v>5.81238880910395</v>
+        <v>2.79478334306542</v>
       </c>
       <c r="D42" t="n">
-        <v>0.0000825116778978451</v>
+        <v>0.445398546415049</v>
       </c>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1125,10 +1125,10 @@
         <v>7</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.000000000566090626090861</v>
+        <v>0.000000000883948171743894</v>
       </c>
       <c r="D43" t="n">
-        <v>0.505982233811905</v>
+        <v>0.679965953342113</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1142,10 +1142,10 @@
         <v>8</v>
       </c>
       <c r="C44" t="n">
-        <v>0.00000000145003879783614</v>
+        <v>-0.00000000191023815189937</v>
       </c>
       <c r="D44" t="n">
-        <v>0.529474482582183</v>
+        <v>0.410448185501649</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1159,10 +1159,10 @@
         <v>9</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.000000000460199354064738</v>
+        <v>-0.00000000223216820128062</v>
       </c>
       <c r="D45" t="n">
-        <v>0.708423320257072</v>
+        <v>0.330908450988018</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1176,10 +1176,10 @@
         <v>10</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.000000000782129403445355</v>
+        <v>-0.00000000145003879783463</v>
       </c>
       <c r="D46" t="n">
-        <v>0.508242214238436</v>
+        <v>0.529474482582666</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1193,10 +1193,10 @@
         <v>6</v>
       </c>
       <c r="C47" t="n">
-        <v>-2.20646450300228</v>
+        <v>0.236758486903971</v>
       </c>
       <c r="D47" t="n">
-        <v>0.359422288023277</v>
+        <v>0.968698351973054</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1210,10 +1210,10 @@
         <v>7</v>
       </c>
       <c r="C48" t="n">
-        <v>0.00000000251319006597743</v>
+        <v>0.00000000100896816679364</v>
       </c>
       <c r="D48" t="n">
-        <v>0.07376588553729</v>
+        <v>0.775100128931755</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1227,10 +1227,10 @@
         <v>8</v>
       </c>
       <c r="C49" t="n">
-        <v>-0.00000000150422189918341</v>
+        <v>0.00000000223382553823967</v>
       </c>
       <c r="D49" t="n">
-        <v>0.692210401454423</v>
+        <v>0.559109396988418</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1244,10 +1244,10 @@
         <v>9</v>
       </c>
       <c r="C50" t="n">
-        <v>0.00000000072960363905609</v>
+        <v>-0.0000000018250625699334</v>
       </c>
       <c r="D50" t="n">
-        <v>0.719034910278691</v>
+        <v>0.629385052065998</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1261,10 +1261,10 @@
         <v>10</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.0000000033292844691178</v>
+        <v>0.00000000150422189918424</v>
       </c>
       <c r="D51" t="n">
-        <v>0.0880706673223342</v>
+        <v>0.692210401454301</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1278,13 +1278,13 @@
         <v>6</v>
       </c>
       <c r="C52" t="n">
-        <v>-12.114279957887</v>
+        <v>-0.520289787879494</v>
       </c>
       <c r="D52" t="n">
-        <v>0.00587195039090193</v>
+        <v>0.962160263692462</v>
       </c>
       <c r="E52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1295,13 +1295,13 @@
         <v>7</v>
       </c>
       <c r="C53" t="n">
-        <v>0.00000000794454840900081</v>
+        <v>0.000000000498245028080136</v>
       </c>
       <c r="D53" t="n">
-        <v>0.00196536814246602</v>
+        <v>0.938125501084188</v>
       </c>
       <c r="E53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1312,10 +1312,10 @@
         <v>8</v>
       </c>
       <c r="C54" t="n">
-        <v>-0.00000000744630338090334</v>
+        <v>-0.00000000244094382394173</v>
       </c>
       <c r="D54" t="n">
-        <v>0.281335402517086</v>
+        <v>0.725407765995985</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1329,13 +1329,13 @@
         <v>9</v>
       </c>
       <c r="C55" t="n">
-        <v>-0.00000000988724720486532</v>
+        <v>-0.0000000023242925750963</v>
       </c>
       <c r="D55" t="n">
-        <v>0.0076155180729657</v>
+        <v>0.735241858941042</v>
       </c>
       <c r="E55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -1346,13 +1346,13 @@
         <v>10</v>
       </c>
       <c r="C56" t="n">
-        <v>-0.00000000977059595601683</v>
+        <v>0.00000000744630338092298</v>
       </c>
       <c r="D56" t="n">
-        <v>0.00605506243492813</v>
+        <v>0.281335402515882</v>
       </c>
       <c r="E56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>